<commit_message>
feat: add pivot-style summaries per ART/team
- New Summary_ART and Summary_Team sheets generated with SUMIF/SUMIFS formulas
- Aggregates headcount, capacity, per-sprint hours, totals, utilization, over/under
- README updated accordingly
</commit_message>
<xml_diff>
--- a/ACME_Project_Team_Workload.xlsx
+++ b/ACME_Project_Team_Workload.xlsx
@@ -16,7 +16,9 @@
     <sheet name="RACI" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Risks_Issues" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Resource_Workload" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Dashboard" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Summary_ART" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Summary_Team" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Dashboard" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,6 +539,1697 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ART</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Headcount</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Cap/Sprint</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>S1 Hrs</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>S2 Hrs</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>S3 Hrs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>S4 Hrs</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>S5 Hrs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>S6 Hrs</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>S7 Hrs</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>S8 Hrs</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Overall Util %</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Util %</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under Hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ART 1</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A2)</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>IFERROR(L2/(C2*8),0)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>SUMIF(Resource_Workload!$D:$D,$A2,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ART 2</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A3)</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M3">
+        <f>IFERROR(L3/(C3*8),0)</f>
+        <v/>
+      </c>
+      <c r="N3">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O3">
+        <f>SUMIF(Resource_Workload!$D:$D,$A3,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ART 3</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A4)</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M4">
+        <f>IFERROR(L4/(C4*8),0)</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O4">
+        <f>SUMIF(Resource_Workload!$D:$D,$A4,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ART 4</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A5)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>IFERROR(L5/(C5*8),0)</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O5">
+        <f>SUMIF(Resource_Workload!$D:$D,$A5,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ART 5</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A6)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M6">
+        <f>IFERROR(L6/(C6*8),0)</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O6">
+        <f>SUMIF(Resource_Workload!$D:$D,$A6,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ART 6</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A7)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M7">
+        <f>IFERROR(L7/(C7*8),0)</f>
+        <v/>
+      </c>
+      <c r="N7">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O7">
+        <f>SUMIF(Resource_Workload!$D:$D,$A7,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ART 7</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Resource_Workload!$D:$D,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$P:$P)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$Q:$Q)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$R:$R)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$S:$S)</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$T:$T)</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$U:$U)</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$V:$V)</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$W:$W)</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$X:$X)</f>
+        <v/>
+      </c>
+      <c r="M8">
+        <f>IFERROR(L8/(C8*8),0)</f>
+        <v/>
+      </c>
+      <c r="N8">
+        <f>AVERAGEIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$Y:$Y)</f>
+        <v/>
+      </c>
+      <c r="O8">
+        <f>SUMIF(Resource_Workload!$D:$D,$A8,Resource_Workload!$Z:$Z)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ART</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Headcount</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Cap/Sprint</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>S1 Hrs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>S2 Hrs</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>S3 Hrs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>S4 Hrs</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>S5 Hrs</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>S6 Hrs</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>S7 Hrs</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>S8 Hrs</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Total Hrs</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Overall Util %</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Util %</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Over/Under Hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ART 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Justice League Command</t>
+        </is>
+      </c>
+      <c r="D2">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="N2">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="O2">
+        <f>IFERROR(N2/(E2*8),0)</f>
+        <v/>
+      </c>
+      <c r="P2">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+      <c r="Q2">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A2,Resource_Workload!$E:$E,$B2,Resource_Workload!$F:$F,$C2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ART 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Avengers Interface</t>
+        </is>
+      </c>
+      <c r="D3">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="L3">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="M3">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="N3">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="O3">
+        <f>IFERROR(N3/(E3*8),0)</f>
+        <v/>
+      </c>
+      <c r="P3">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+      <c r="Q3">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A3,Resource_Workload!$E:$E,$B3,Resource_Workload!$F:$F,$C3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ART 2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>X-Men Flight</t>
+        </is>
+      </c>
+      <c r="D4">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="M4">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="O4">
+        <f>IFERROR(N4/(E4*8),0)</f>
+        <v/>
+      </c>
+      <c r="P4">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+      <c r="Q4">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A4,Resource_Workload!$E:$E,$B4,Resource_Workload!$F:$F,$C4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ART 2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Fantastic Four Navigation</t>
+        </is>
+      </c>
+      <c r="D5">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="O5">
+        <f>IFERROR(N5/(E5*8),0)</f>
+        <v/>
+      </c>
+      <c r="P5">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+      <c r="Q5">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A5,Resource_Workload!$E:$E,$B5,Resource_Workload!$F:$F,$C5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ART 3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Teen Titans Communication</t>
+        </is>
+      </c>
+      <c r="D6">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="M6">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="O6">
+        <f>IFERROR(N6/(E6*8),0)</f>
+        <v/>
+      </c>
+      <c r="P6">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+      <c r="Q6">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A6,Resource_Workload!$E:$E,$B6,Resource_Workload!$F:$F,$C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ART 3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Guardians of the Network</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="M7">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="N7">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="O7">
+        <f>IFERROR(N7/(E7*8),0)</f>
+        <v/>
+      </c>
+      <c r="P7">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+      <c r="Q7">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A7,Resource_Workload!$E:$E,$B7,Resource_Workload!$F:$F,$C7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ART 4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>S.H.I.E.L.D. Security</t>
+        </is>
+      </c>
+      <c r="D8">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="M8">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="N8">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="O8">
+        <f>IFERROR(N8/(E8*8),0)</f>
+        <v/>
+      </c>
+      <c r="P8">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+      <c r="Q8">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A8,Resource_Workload!$E:$E,$B8,Resource_Workload!$F:$F,$C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ART 4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Watchmen Intrusion</t>
+        </is>
+      </c>
+      <c r="D9">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="N9">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="O9">
+        <f>IFERROR(N9/(E9*8),0)</f>
+        <v/>
+      </c>
+      <c r="P9">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+      <c r="Q9">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A9,Resource_Workload!$E:$E,$B9,Resource_Workload!$F:$F,$C9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ART 5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Avengers Intelligence</t>
+        </is>
+      </c>
+      <c r="D10">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="L10">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="M10">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="N10">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="O10">
+        <f>IFERROR(N10/(E10*8),0)</f>
+        <v/>
+      </c>
+      <c r="P10">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+      <c r="Q10">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A10,Resource_Workload!$E:$E,$B10,Resource_Workload!$F:$F,$C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ART 5</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Justice League Analytics</t>
+        </is>
+      </c>
+      <c r="D11">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="L11">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="M11">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="N11">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="O11">
+        <f>IFERROR(N11/(E11*8),0)</f>
+        <v/>
+      </c>
+      <c r="P11">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+      <c r="Q11">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A11,Resource_Workload!$E:$E,$B11,Resource_Workload!$F:$F,$C11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ART 6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>X-Men Coordination</t>
+        </is>
+      </c>
+      <c r="D12">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="L12">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="M12">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="N12">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="O12">
+        <f>IFERROR(N12/(E12*8),0)</f>
+        <v/>
+      </c>
+      <c r="P12">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+      <c r="Q12">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A12,Resource_Workload!$E:$E,$B12,Resource_Workload!$F:$F,$C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ART 6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fantastic Four Intelligence</t>
+        </is>
+      </c>
+      <c r="D13">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="M13">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="N13">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="O13">
+        <f>IFERROR(N13/(E13*8),0)</f>
+        <v/>
+      </c>
+      <c r="P13">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+      <c r="Q13">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A13,Resource_Workload!$E:$E,$B13,Resource_Workload!$F:$F,$C13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ART 7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Team Alpha</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Avengers Assembly</t>
+        </is>
+      </c>
+      <c r="D14">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="K14">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="L14">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="M14">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="N14">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="O14">
+        <f>IFERROR(N14/(E14*8),0)</f>
+        <v/>
+      </c>
+      <c r="P14">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+      <c r="Q14">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A14,Resource_Workload!$E:$E,$B14,Resource_Workload!$F:$F,$C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ART 7</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Team Beta</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Justice League Validation</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS(Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>SUMIFS(Resource_Workload!$G:$G,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>SUMIFS(Resource_Workload!$P:$P,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>SUMIFS(Resource_Workload!$Q:$Q,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>SUMIFS(Resource_Workload!$R:$R,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>SUMIFS(Resource_Workload!$S:$S,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>SUMIFS(Resource_Workload!$T:$T,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="K15">
+        <f>SUMIFS(Resource_Workload!$U:$U,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="L15">
+        <f>SUMIFS(Resource_Workload!$V:$V,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="M15">
+        <f>SUMIFS(Resource_Workload!$W:$W,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="N15">
+        <f>SUMIFS(Resource_Workload!$X:$X,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="O15">
+        <f>IFERROR(N15/(E15*8),0)</f>
+        <v/>
+      </c>
+      <c r="P15">
+        <f>AVERAGEIFS(Resource_Workload!$Y:$Y,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+      <c r="Q15">
+        <f>SUMIFS(Resource_Workload!$Z:$Z,Resource_Workload!$D:$D,$A15,Resource_Workload!$E:$E,$B15,Resource_Workload!$F:$F,$C15)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
feat: import tasks CSV and roll up actual hours per assignee
- Add --tasks-csv flag
- Create Actual_Tasks and Actuals_Rollup sheets
- Add Summary_Actuals_ART and Summary_Actuals_Team aggregates
- Keep planned sheets intact; skip actuals if no CSV is provided
- Update README with CSV schema and usage
</commit_message>
<xml_diff>
--- a/ACME_Project_Team_Workload.xlsx
+++ b/ACME_Project_Team_Workload.xlsx
@@ -2375,8 +2375,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2419,8 +2417,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2463,8 +2459,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2507,8 +2501,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2551,8 +2543,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2595,8 +2585,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2639,8 +2627,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2683,8 +2669,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2727,8 +2711,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2771,8 +2753,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2815,8 +2795,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2859,8 +2837,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2903,8 +2879,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2947,8 +2921,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2991,8 +2963,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3035,8 +3005,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3079,8 +3047,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3123,8 +3089,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3167,8 +3131,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3211,8 +3173,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3255,8 +3215,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3299,8 +3257,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3343,8 +3299,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3387,8 +3341,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3431,8 +3383,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3475,8 +3425,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3519,8 +3467,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3563,8 +3509,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3607,8 +3551,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3651,8 +3593,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3695,8 +3635,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3739,8 +3677,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3783,8 +3719,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3827,8 +3761,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3871,8 +3803,6 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3976,7 +3906,6 @@
           <t>Batman</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4014,7 +3943,6 @@
           <t>Superman</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4052,7 +3980,6 @@
           <t>Wonder Woman</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4090,7 +4017,6 @@
           <t>Iron Man</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4128,7 +4054,6 @@
           <t>Captain America</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4166,7 +4091,6 @@
           <t>Professor X</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4204,7 +4128,6 @@
           <t>Cyclops</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4242,7 +4165,6 @@
           <t>Storm</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4280,7 +4202,6 @@
           <t>Reed Richards</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4318,7 +4239,6 @@
           <t>Sue Storm</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4356,7 +4276,6 @@
           <t>Raven</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4394,7 +4313,6 @@
           <t>Robin</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4432,7 +4350,6 @@
           <t>Cyborg</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4470,7 +4387,6 @@
           <t>Star-Lord</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4508,7 +4424,6 @@
           <t>Rocket</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4546,7 +4461,6 @@
           <t>Nick Fury</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4584,7 +4498,6 @@
           <t>Black Widow</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4622,7 +4535,6 @@
           <t>Doctor Strange</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4660,7 +4572,6 @@
           <t>Rorschach</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4698,7 +4609,6 @@
           <t>Ozymandias</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4736,7 +4646,6 @@
           <t>Vision</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4774,7 +4683,6 @@
           <t>Hawkeye</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4812,7 +4720,6 @@
           <t>Scarlet Witch</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4850,7 +4757,6 @@
           <t>Martian Manhunter</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4888,7 +4794,6 @@
           <t>Green Lantern</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4926,7 +4831,6 @@
           <t>Jean Grey</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4964,7 +4868,6 @@
           <t>Wolverine</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5002,7 +4905,6 @@
           <t>Magneto</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5040,7 +4942,6 @@
           <t>Reed Richards</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5078,7 +4979,6 @@
           <t>Thing</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5116,7 +5016,6 @@
           <t>Thor</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5154,7 +5053,6 @@
           <t>Hulk</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5192,7 +5090,6 @@
           <t>Ant-Man</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5230,7 +5127,6 @@
           <t>Flash</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5268,7 +5164,6 @@
           <t>Aquaman</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5306,7 +5201,6 @@
           <t>Clint Barton</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5344,7 +5238,6 @@
           <t>Dane Whitman</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5382,7 +5275,6 @@
           <t>Nebula</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5420,7 +5312,6 @@
           <t>Yelena Belova</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5458,7 +5349,6 @@
           <t>Kate Bishop</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5496,7 +5386,6 @@
           <t>Peter Parker</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5534,7 +5423,6 @@
           <t>Luke Cage</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5572,7 +5460,6 @@
           <t>Sam Wilson</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5610,7 +5497,6 @@
           <t>Gamora</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5648,7 +5534,6 @@
           <t>Monica Rambeau</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5686,7 +5571,6 @@
           <t>Ben Grimm</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5724,7 +5608,6 @@
           <t>Maria Hill</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5762,7 +5645,6 @@
           <t>Matt Murdock</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5800,7 +5682,6 @@
           <t>Stephen Strange</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5838,7 +5719,6 @@
           <t>Pepper Potts</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5876,7 +5756,6 @@
           <t>Carol Danvers</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5914,7 +5793,6 @@
           <t>Jessica Jones</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5952,7 +5830,6 @@
           <t>Quake Johnson</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5990,7 +5867,6 @@
           <t>Bucky Barnes</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6028,7 +5904,6 @@
           <t>Tony Stark</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6066,7 +5941,6 @@
           <t>Frank Castle</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6104,7 +5978,6 @@
           <t>T'Challa</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6142,7 +6015,6 @@
           <t>Steve Rogers</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6180,7 +6052,6 @@
           <t>Shang-Chi</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6218,7 +6089,6 @@
           <t>Rene Ramirez</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6256,7 +6126,6 @@
           <t>Tim Drake</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6294,7 +6163,6 @@
           <t>Helena Bertinelli</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6332,7 +6200,6 @@
           <t>Dinah Lance</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6370,7 +6237,6 @@
           <t>Stephanie Brown</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6408,7 +6274,6 @@
           <t>Kendra Saunders</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6446,7 +6311,6 @@
           <t>Mari McCabe</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6484,7 +6348,6 @@
           <t>Victor Zsasz</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6522,7 +6385,6 @@
           <t>Carter Hall</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6560,7 +6422,6 @@
           <t>John Stewart</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6598,7 +6459,6 @@
           <t>Zatanna Zatara</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6636,7 +6496,6 @@
           <t>Kaldur'ahm</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6674,7 +6533,6 @@
           <t>Ryan Choi</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6712,7 +6570,6 @@
           <t>Donna Troy</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6750,7 +6607,6 @@
           <t>Eobard Thawne</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6788,7 +6644,6 @@
           <t>Barbara Gordon</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6826,7 +6681,6 @@
           <t>Shuri</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6864,7 +6718,6 @@
           <t>Danny Rand</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6902,7 +6755,6 @@
           <t>Johnny Storm</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6940,7 +6792,6 @@
           <t>Bruce Banner</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6978,7 +6829,6 @@
           <t>Groot</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7016,7 +6866,6 @@
           <t>Okoye</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7054,7 +6903,6 @@
           <t>Hank Pym</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7092,7 +6940,6 @@
           <t>Jennifer Walters</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7130,7 +6977,6 @@
           <t>Rory Regan</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7168,7 +7014,6 @@
           <t>Huntress Wayne</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7206,7 +7051,6 @@
           <t>Oliver Queen</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7244,7 +7088,6 @@
           <t>Ravager Wilson</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7282,7 +7125,6 @@
           <t>Cassandra Cain</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7320,7 +7162,6 @@
           <t>Kara Zor-El</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7358,7 +7199,6 @@
           <t>Wally West</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7396,7 +7236,6 @@
           <t>Talia al Ghul</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9836,7 +9675,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -9925,7 +9764,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -10014,7 +9853,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -10103,7 +9942,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -10192,7 +10031,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -10281,7 +10120,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -10370,7 +10209,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -10459,7 +10298,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -10548,7 +10387,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -10637,7 +10476,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -10726,7 +10565,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -10815,7 +10654,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -10904,7 +10743,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -10993,7 +10832,7 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -11082,7 +10921,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -11171,7 +11010,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -11260,7 +11099,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -11349,7 +11188,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -11438,7 +11277,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -11527,7 +11366,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -11616,7 +11455,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -11705,7 +11544,7 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -11794,7 +11633,7 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -11883,7 +11722,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -11972,7 +11811,7 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -12061,7 +11900,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -12150,7 +11989,7 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -12239,7 +12078,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -12328,7 +12167,7 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -12417,7 +12256,7 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -12506,7 +12345,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -12595,7 +12434,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -12684,7 +12523,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -12773,7 +12612,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -12862,7 +12701,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -12951,7 +12790,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -13040,7 +12879,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -13129,7 +12968,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -13218,7 +13057,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -13307,7 +13146,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -13396,7 +13235,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -13485,7 +13324,7 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -13574,7 +13413,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -13663,7 +13502,7 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -13752,7 +13591,7 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -13841,7 +13680,7 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -13930,7 +13769,7 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -14019,7 +13858,7 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -14108,7 +13947,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -14197,7 +14036,7 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -14286,7 +14125,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -14375,7 +14214,7 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H53" t="n">
         <v>0</v>
@@ -14464,7 +14303,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H54" t="n">
         <v>0</v>
@@ -14553,7 +14392,7 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H55" t="n">
         <v>0</v>
@@ -14642,7 +14481,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -14731,7 +14570,7 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -14820,7 +14659,7 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -14909,7 +14748,7 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H59" t="n">
         <v>0</v>
@@ -14998,7 +14837,7 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H60" t="n">
         <v>0</v>
@@ -15087,7 +14926,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H61" t="n">
         <v>0</v>
@@ -15176,7 +15015,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -15265,7 +15104,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -15354,7 +15193,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -15443,7 +15282,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -15532,7 +15371,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -15621,7 +15460,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -15710,7 +15549,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -15799,7 +15638,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -15888,7 +15727,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -15977,7 +15816,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -16066,7 +15905,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H72" t="n">
         <v>0</v>
@@ -16155,7 +15994,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -16244,7 +16083,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -16333,7 +16172,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>
@@ -16422,7 +16261,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H76" t="n">
         <v>0</v>
@@ -16511,7 +16350,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
@@ -16600,7 +16439,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
@@ -16689,7 +16528,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H79" t="n">
         <v>0</v>
@@ -16778,7 +16617,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H80" t="n">
         <v>0</v>
@@ -16867,7 +16706,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H81" t="n">
         <v>0</v>
@@ -16956,7 +16795,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H82" t="n">
         <v>0</v>
@@ -17045,7 +16884,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H83" t="n">
         <v>0</v>
@@ -17134,7 +16973,7 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H84" t="n">
         <v>0</v>
@@ -17223,7 +17062,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H85" t="n">
         <v>0</v>
@@ -17312,7 +17151,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H86" t="n">
         <v>0</v>
@@ -17401,7 +17240,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H87" t="n">
         <v>0</v>
@@ -17490,7 +17329,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
@@ -17579,7 +17418,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H89" t="n">
         <v>0</v>
@@ -17668,7 +17507,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H90" t="n">
         <v>0</v>
@@ -17757,7 +17596,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H91" t="n">
         <v>0</v>
@@ -17846,7 +17685,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H92" t="n">
         <v>0</v>

</xml_diff>